<commit_message>
Fix date format in weights Excel — plain strings instead of timestamps
</commit_message>
<xml_diff>
--- a/Data/outputs/v2_portfolio_weights.xlsx
+++ b/Data/outputs/v2_portfolio_weights.xlsx
@@ -16,10 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -648,8 +644,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>40268</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2010-03-31</t>
+        </is>
       </c>
       <c r="B2" t="n">
         <v>0.06</v>
@@ -785,8 +783,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>40298</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2010-04-30</t>
+        </is>
       </c>
       <c r="B3" t="n">
         <v>0.06</v>
@@ -922,8 +922,10 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>40359</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2010-06-30</t>
+        </is>
       </c>
       <c r="B4" t="n">
         <v>0</v>
@@ -1059,8 +1061,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>40421</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2010-08-31</t>
+        </is>
       </c>
       <c r="B5" t="n">
         <v>0</v>
@@ -1196,8 +1200,10 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>40451</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2010-09-30</t>
+        </is>
       </c>
       <c r="B6" t="n">
         <v>0</v>
@@ -1333,8 +1339,10 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>40512</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2010-11-30</t>
+        </is>
       </c>
       <c r="B7" t="n">
         <v>0.06</v>
@@ -1470,8 +1478,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>40543</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2010-12-31</t>
+        </is>
       </c>
       <c r="B8" t="n">
         <v>0.06</v>
@@ -1607,8 +1617,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>40574</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2011-01-31</t>
+        </is>
       </c>
       <c r="B9" t="n">
         <v>0.06</v>
@@ -1744,8 +1756,10 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>40602</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2011-02-28</t>
+        </is>
       </c>
       <c r="B10" t="n">
         <v>0.06</v>
@@ -1881,8 +1895,10 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>40633</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2011-03-31</t>
+        </is>
       </c>
       <c r="B11" t="n">
         <v>0.0801</v>
@@ -2018,8 +2034,10 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>40694</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2011-05-31</t>
+        </is>
       </c>
       <c r="B12" t="n">
         <v>0.0117</v>
@@ -2155,8 +2173,10 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>40724</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2011-06-30</t>
+        </is>
       </c>
       <c r="B13" t="n">
         <v>0</v>
@@ -2292,8 +2312,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>40786</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2011-08-31</t>
+        </is>
       </c>
       <c r="B14" t="n">
         <v>0</v>
@@ -2429,8 +2451,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>40816</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2011-09-30</t>
+        </is>
       </c>
       <c r="B15" t="n">
         <v>0</v>
@@ -2566,8 +2590,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>40847</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2011-10-31</t>
+        </is>
       </c>
       <c r="B16" t="n">
         <v>0.3177</v>
@@ -2703,8 +2729,10 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>40877</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2011-11-30</t>
+        </is>
       </c>
       <c r="B17" t="n">
         <v>0</v>
@@ -2840,8 +2868,10 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>40939</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2012-01-31</t>
+        </is>
       </c>
       <c r="B18" t="n">
         <v>0.155</v>
@@ -2977,8 +3007,10 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>40968</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2012-02-29</t>
+        </is>
       </c>
       <c r="B19" t="n">
         <v>0</v>
@@ -3114,8 +3146,10 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>41029</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2012-04-30</t>
+        </is>
       </c>
       <c r="B20" t="n">
         <v>0</v>
@@ -3251,8 +3285,10 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>41060</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2012-05-31</t>
+        </is>
       </c>
       <c r="B21" t="n">
         <v>0</v>
@@ -3388,8 +3424,10 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>41121</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2012-07-31</t>
+        </is>
       </c>
       <c r="B22" t="n">
         <v>0</v>
@@ -3525,8 +3563,10 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>41152</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2012-08-31</t>
+        </is>
       </c>
       <c r="B23" t="n">
         <v>0</v>
@@ -3662,8 +3702,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>41213</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2012-10-31</t>
+        </is>
       </c>
       <c r="B24" t="n">
         <v>0.06</v>
@@ -3799,8 +3841,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>41243</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2012-11-30</t>
+        </is>
       </c>
       <c r="B25" t="n">
         <v>0</v>
@@ -3936,8 +3980,10 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>41274</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2012-12-31</t>
+        </is>
       </c>
       <c r="B26" t="n">
         <v>0.06</v>
@@ -4073,8 +4119,10 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>41305</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2013-01-31</t>
+        </is>
       </c>
       <c r="B27" t="n">
         <v>0.06</v>
@@ -4210,8 +4258,10 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
-        <v>41333</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2013-02-28</t>
+        </is>
       </c>
       <c r="B28" t="n">
         <v>0.06</v>
@@ -4347,8 +4397,10 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
-        <v>41394</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2013-04-30</t>
+        </is>
       </c>
       <c r="B29" t="n">
         <v>0</v>
@@ -4484,8 +4536,10 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
-        <v>41425</v>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2013-05-31</t>
+        </is>
       </c>
       <c r="B30" t="n">
         <v>0.06</v>
@@ -4621,8 +4675,10 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
-        <v>41486</v>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2013-07-31</t>
+        </is>
       </c>
       <c r="B31" t="n">
         <v>0.06</v>
@@ -4758,8 +4814,10 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
-        <v>41547</v>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2013-09-30</t>
+        </is>
       </c>
       <c r="B32" t="n">
         <v>0.06</v>
@@ -4895,8 +4953,10 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
-        <v>41578</v>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2013-10-31</t>
+        </is>
       </c>
       <c r="B33" t="n">
         <v>0</v>
@@ -5032,8 +5092,10 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
-        <v>41639</v>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2013-12-31</t>
+        </is>
       </c>
       <c r="B34" t="n">
         <v>0.06</v>
@@ -5169,8 +5231,10 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
-        <v>41670</v>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2014-01-31</t>
+        </is>
       </c>
       <c r="B35" t="n">
         <v>0</v>
@@ -5306,8 +5370,10 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
-        <v>41698</v>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2014-02-28</t>
+        </is>
       </c>
       <c r="B36" t="n">
         <v>0</v>
@@ -5443,8 +5509,10 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
-        <v>41729</v>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2014-03-31</t>
+        </is>
       </c>
       <c r="B37" t="n">
         <v>0</v>
@@ -5580,8 +5648,10 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
-        <v>41759</v>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2014-04-30</t>
+        </is>
       </c>
       <c r="B38" t="n">
         <v>0</v>
@@ -5717,8 +5787,10 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
-        <v>41820</v>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2014-06-30</t>
+        </is>
       </c>
       <c r="B39" t="n">
         <v>0</v>
@@ -5854,8 +5926,10 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
-        <v>41851</v>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2014-07-31</t>
+        </is>
       </c>
       <c r="B40" t="n">
         <v>0</v>
@@ -5991,8 +6065,10 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
-        <v>41912</v>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2014-09-30</t>
+        </is>
       </c>
       <c r="B41" t="n">
         <v>0.06</v>
@@ -6128,8 +6204,10 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
-        <v>41943</v>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2014-10-31</t>
+        </is>
       </c>
       <c r="B42" t="n">
         <v>0</v>
@@ -6265,8 +6343,10 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
-        <v>42004</v>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2014-12-31</t>
+        </is>
       </c>
       <c r="B43" t="n">
         <v>0</v>
@@ -6402,8 +6482,10 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
-        <v>42094</v>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2015-03-31</t>
+        </is>
       </c>
       <c r="B44" t="n">
         <v>0</v>
@@ -6539,8 +6621,10 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
-        <v>42124</v>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2015-04-30</t>
+        </is>
       </c>
       <c r="B45" t="n">
         <v>0</v>
@@ -6676,8 +6760,10 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
-        <v>42185</v>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2015-06-30</t>
+        </is>
       </c>
       <c r="B46" t="n">
         <v>0.06</v>
@@ -6813,8 +6899,10 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>42216</v>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2015-07-31</t>
+        </is>
       </c>
       <c r="B47" t="n">
         <v>0.06</v>
@@ -6950,8 +7038,10 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
-        <v>42247</v>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2015-08-31</t>
+        </is>
       </c>
       <c r="B48" t="n">
         <v>0</v>
@@ -7087,8 +7177,10 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>42277</v>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2015-09-30</t>
+        </is>
       </c>
       <c r="B49" t="n">
         <v>0</v>
@@ -7224,8 +7316,10 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
-        <v>42338</v>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2015-11-30</t>
+        </is>
       </c>
       <c r="B50" t="n">
         <v>0.06</v>
@@ -7361,8 +7455,10 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
-        <v>42369</v>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2015-12-31</t>
+        </is>
       </c>
       <c r="B51" t="n">
         <v>0.06</v>
@@ -7498,8 +7594,10 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
-        <v>42429</v>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2016-02-29</t>
+        </is>
       </c>
       <c r="B52" t="n">
         <v>0</v>
@@ -7635,8 +7733,10 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>42460</v>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2016-03-31</t>
+        </is>
       </c>
       <c r="B53" t="n">
         <v>0.0505</v>
@@ -7772,8 +7872,10 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
-        <v>42521</v>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2016-05-31</t>
+        </is>
       </c>
       <c r="B54" t="n">
         <v>0</v>
@@ -7909,8 +8011,10 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
-        <v>42551</v>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2016-06-30</t>
+        </is>
       </c>
       <c r="B55" t="n">
         <v>0</v>
@@ -8046,8 +8150,10 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
-        <v>42613</v>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2016-08-31</t>
+        </is>
       </c>
       <c r="B56" t="n">
         <v>0</v>
@@ -8183,8 +8289,10 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
-        <v>42643</v>
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2016-09-30</t>
+        </is>
       </c>
       <c r="B57" t="n">
         <v>0</v>
@@ -8320,8 +8428,10 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
-        <v>42674</v>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2016-10-31</t>
+        </is>
       </c>
       <c r="B58" t="n">
         <v>0.06</v>
@@ -8457,8 +8567,10 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
-        <v>42704</v>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2016-11-30</t>
+        </is>
       </c>
       <c r="B59" t="n">
         <v>0.06</v>
@@ -8594,8 +8706,10 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
-        <v>42766</v>
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2017-01-31</t>
+        </is>
       </c>
       <c r="B60" t="n">
         <v>0.06</v>
@@ -8731,8 +8845,10 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
-        <v>42794</v>
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2017-02-28</t>
+        </is>
       </c>
       <c r="B61" t="n">
         <v>0.06</v>
@@ -8868,8 +8984,10 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
-        <v>42825</v>
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2017-03-31</t>
+        </is>
       </c>
       <c r="B62" t="n">
         <v>0</v>
@@ -9005,8 +9123,10 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
-        <v>42886</v>
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2017-05-31</t>
+        </is>
       </c>
       <c r="B63" t="n">
         <v>0</v>
@@ -9142,8 +9262,10 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
-        <v>42916</v>
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2017-06-30</t>
+        </is>
       </c>
       <c r="B64" t="n">
         <v>0</v>
@@ -9279,8 +9401,10 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
-        <v>42947</v>
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2017-07-31</t>
+        </is>
       </c>
       <c r="B65" t="n">
         <v>0</v>
@@ -9416,8 +9540,10 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
-        <v>42978</v>
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2017-08-31</t>
+        </is>
       </c>
       <c r="B66" t="n">
         <v>0</v>
@@ -9553,8 +9679,10 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
-        <v>43039</v>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2017-10-31</t>
+        </is>
       </c>
       <c r="B67" t="n">
         <v>0.06</v>
@@ -9690,8 +9818,10 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
-        <v>43069</v>
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2017-11-30</t>
+        </is>
       </c>
       <c r="B68" t="n">
         <v>0</v>
@@ -9827,8 +9957,10 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
-        <v>43131</v>
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2018-01-31</t>
+        </is>
       </c>
       <c r="B69" t="n">
         <v>0.06</v>
@@ -9964,8 +10096,10 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
-        <v>43159</v>
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2018-02-28</t>
+        </is>
       </c>
       <c r="B70" t="n">
         <v>0.06</v>
@@ -10101,8 +10235,10 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
-        <v>43220</v>
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2018-04-30</t>
+        </is>
       </c>
       <c r="B71" t="n">
         <v>0.06</v>
@@ -10238,8 +10374,10 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
-        <v>43251</v>
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2018-05-31</t>
+        </is>
       </c>
       <c r="B72" t="n">
         <v>0</v>
@@ -10375,8 +10513,10 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
-        <v>43312</v>
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2018-07-31</t>
+        </is>
       </c>
       <c r="B73" t="n">
         <v>0.06</v>
@@ -10512,8 +10652,10 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
-        <v>43343</v>
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2018-08-31</t>
+        </is>
       </c>
       <c r="B74" t="n">
         <v>0</v>
@@ -10649,8 +10791,10 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
-        <v>43404</v>
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2018-10-31</t>
+        </is>
       </c>
       <c r="B75" t="n">
         <v>0.15</v>
@@ -10786,8 +10930,10 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
-        <v>43434</v>
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2018-11-30</t>
+        </is>
       </c>
       <c r="B76" t="n">
         <v>0</v>
@@ -10923,8 +11069,10 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
-        <v>43465</v>
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2018-12-31</t>
+        </is>
       </c>
       <c r="B77" t="n">
         <v>0</v>
@@ -11060,8 +11208,10 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
-        <v>43496</v>
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2019-01-31</t>
+        </is>
       </c>
       <c r="B78" t="n">
         <v>0</v>
@@ -11197,8 +11347,10 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
-        <v>43524</v>
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2019-02-28</t>
+        </is>
       </c>
       <c r="B79" t="n">
         <v>0</v>
@@ -11334,8 +11486,10 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
-        <v>43585</v>
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2019-04-30</t>
+        </is>
       </c>
       <c r="B80" t="n">
         <v>0</v>
@@ -11471,8 +11625,10 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
-        <v>43616</v>
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2019-05-31</t>
+        </is>
       </c>
       <c r="B81" t="n">
         <v>0</v>
@@ -11608,8 +11764,10 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
-        <v>43677</v>
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2019-07-31</t>
+        </is>
       </c>
       <c r="B82" t="n">
         <v>0</v>
@@ -11745,8 +11903,10 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
-        <v>43738</v>
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2019-09-30</t>
+        </is>
       </c>
       <c r="B83" t="n">
         <v>0</v>
@@ -11882,8 +12042,10 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
-        <v>43769</v>
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2019-10-31</t>
+        </is>
       </c>
       <c r="B84" t="n">
         <v>0</v>
@@ -12019,8 +12181,10 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
-        <v>43830</v>
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2019-12-31</t>
+        </is>
       </c>
       <c r="B85" t="n">
         <v>0.06</v>
@@ -12156,8 +12320,10 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
-        <v>43861</v>
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2020-01-31</t>
+        </is>
       </c>
       <c r="B86" t="n">
         <v>0</v>
@@ -12293,8 +12459,10 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
-        <v>43921</v>
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2020-03-31</t>
+        </is>
       </c>
       <c r="B87" t="n">
         <v>0.4152</v>
@@ -12430,8 +12598,10 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
-        <v>43951</v>
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2020-04-30</t>
+        </is>
       </c>
       <c r="B88" t="n">
         <v>0.485</v>
@@ -12567,8 +12737,10 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
-        <v>44012</v>
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2020-06-30</t>
+        </is>
       </c>
       <c r="B89" t="n">
         <v>0</v>
@@ -12704,8 +12876,10 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
-        <v>44043</v>
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2020-07-31</t>
+        </is>
       </c>
       <c r="B90" t="n">
         <v>0.2503</v>
@@ -12841,8 +13015,10 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
-        <v>44074</v>
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2020-08-31</t>
+        </is>
       </c>
       <c r="B91" t="n">
         <v>0.0674</v>
@@ -12978,8 +13154,10 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
-        <v>44104</v>
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2020-09-30</t>
+        </is>
       </c>
       <c r="B92" t="n">
         <v>0</v>
@@ -13115,8 +13293,10 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="1" t="n">
-        <v>44165</v>
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2020-11-30</t>
+        </is>
       </c>
       <c r="B93" t="n">
         <v>0.1157</v>
@@ -13252,8 +13432,10 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="1" t="n">
-        <v>44196</v>
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2020-12-31</t>
+        </is>
       </c>
       <c r="B94" t="n">
         <v>0.06</v>
@@ -13389,8 +13571,10 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="1" t="n">
-        <v>44286</v>
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2021-03-31</t>
+        </is>
       </c>
       <c r="B95" t="n">
         <v>0.1706</v>
@@ -13526,8 +13710,10 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="1" t="n">
-        <v>44316</v>
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2021-04-30</t>
+        </is>
       </c>
       <c r="B96" t="n">
         <v>0.06</v>
@@ -13663,8 +13849,10 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="1" t="n">
-        <v>44377</v>
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2021-06-30</t>
+        </is>
       </c>
       <c r="B97" t="n">
         <v>0</v>
@@ -13800,8 +13988,10 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="1" t="n">
-        <v>44439</v>
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2021-08-31</t>
+        </is>
       </c>
       <c r="B98" t="n">
         <v>0</v>
@@ -13937,8 +14127,10 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="1" t="n">
-        <v>44469</v>
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2021-09-30</t>
+        </is>
       </c>
       <c r="B99" t="n">
         <v>0.0645</v>
@@ -14074,8 +14266,10 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="1" t="n">
-        <v>44530</v>
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2021-11-30</t>
+        </is>
       </c>
       <c r="B100" t="n">
         <v>0.06</v>
@@ -14211,8 +14405,10 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="1" t="n">
-        <v>44561</v>
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2021-12-31</t>
+        </is>
       </c>
       <c r="B101" t="n">
         <v>0.06</v>
@@ -14348,8 +14544,10 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="1" t="n">
-        <v>44592</v>
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2022-01-31</t>
+        </is>
       </c>
       <c r="B102" t="n">
         <v>0.15</v>
@@ -14485,8 +14683,10 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="1" t="n">
-        <v>44620</v>
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2022-02-28</t>
+        </is>
       </c>
       <c r="B103" t="n">
         <v>0.15</v>
@@ -14622,8 +14822,10 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="1" t="n">
-        <v>44651</v>
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2022-03-31</t>
+        </is>
       </c>
       <c r="B104" t="n">
         <v>0.06</v>
@@ -14759,8 +14961,10 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="1" t="n">
-        <v>44712</v>
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2022-05-31</t>
+        </is>
       </c>
       <c r="B105" t="n">
         <v>0.15</v>
@@ -14896,8 +15100,10 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="1" t="n">
-        <v>44742</v>
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2022-06-30</t>
+        </is>
       </c>
       <c r="B106" t="n">
         <v>0.15</v>
@@ -15033,8 +15239,10 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="1" t="n">
-        <v>44804</v>
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2022-08-31</t>
+        </is>
       </c>
       <c r="B107" t="n">
         <v>0.15</v>
@@ -15170,8 +15378,10 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="1" t="n">
-        <v>44834</v>
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2022-09-30</t>
+        </is>
       </c>
       <c r="B108" t="n">
         <v>0.15</v>
@@ -15307,8 +15517,10 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="1" t="n">
-        <v>44865</v>
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2022-10-31</t>
+        </is>
       </c>
       <c r="B109" t="n">
         <v>0.15</v>
@@ -15444,8 +15656,10 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="1" t="n">
-        <v>44895</v>
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2022-11-30</t>
+        </is>
       </c>
       <c r="B110" t="n">
         <v>0.3835</v>
@@ -15581,8 +15795,10 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="1" t="n">
-        <v>44957</v>
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2023-01-31</t>
+        </is>
       </c>
       <c r="B111" t="n">
         <v>0.0532</v>
@@ -15718,8 +15934,10 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="1" t="n">
-        <v>44985</v>
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2023-02-28</t>
+        </is>
       </c>
       <c r="B112" t="n">
         <v>0.06</v>
@@ -15855,8 +16073,10 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="1" t="n">
-        <v>45016</v>
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2023-03-31</t>
+        </is>
       </c>
       <c r="B113" t="n">
         <v>0</v>
@@ -15992,8 +16212,10 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="1" t="n">
-        <v>45077</v>
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2023-05-31</t>
+        </is>
       </c>
       <c r="B114" t="n">
         <v>0.06</v>
@@ -16129,8 +16351,10 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="1" t="n">
-        <v>45107</v>
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2023-06-30</t>
+        </is>
       </c>
       <c r="B115" t="n">
         <v>0.06</v>
@@ -16266,8 +16490,10 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="1" t="n">
-        <v>45138</v>
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2023-07-31</t>
+        </is>
       </c>
       <c r="B116" t="n">
         <v>0.06</v>
@@ -16403,8 +16629,10 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="1" t="n">
-        <v>45169</v>
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2023-08-31</t>
+        </is>
       </c>
       <c r="B117" t="n">
         <v>0.06</v>
@@ -16540,8 +16768,10 @@
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="1" t="n">
-        <v>45230</v>
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2023-10-31</t>
+        </is>
       </c>
       <c r="B118" t="n">
         <v>0.15</v>
@@ -16677,8 +16907,10 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="1" t="n">
-        <v>45260</v>
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2023-11-30</t>
+        </is>
       </c>
       <c r="B119" t="n">
         <v>0.06</v>
@@ -16814,8 +17046,10 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="1" t="n">
-        <v>45322</v>
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2024-01-31</t>
+        </is>
       </c>
       <c r="B120" t="n">
         <v>0.06</v>
@@ -16951,8 +17185,10 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="1" t="n">
-        <v>45351</v>
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2024-02-29</t>
+        </is>
       </c>
       <c r="B121" t="n">
         <v>0.06</v>
@@ -17088,8 +17324,10 @@
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="1" t="n">
-        <v>45412</v>
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2024-04-30</t>
+        </is>
       </c>
       <c r="B122" t="n">
         <v>0.06</v>
@@ -17225,8 +17463,10 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="1" t="n">
-        <v>45443</v>
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2024-05-31</t>
+        </is>
       </c>
       <c r="B123" t="n">
         <v>0.06</v>
@@ -17362,8 +17602,10 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="1" t="n">
-        <v>45504</v>
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2024-07-31</t>
+        </is>
       </c>
       <c r="B124" t="n">
         <v>0</v>
@@ -17499,8 +17741,10 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="1" t="n">
-        <v>45565</v>
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2024-09-30</t>
+        </is>
       </c>
       <c r="B125" t="n">
         <v>0</v>
@@ -17636,8 +17880,10 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="1" t="n">
-        <v>45596</v>
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2024-10-31</t>
+        </is>
       </c>
       <c r="B126" t="n">
         <v>0.06</v>
@@ -17773,8 +18019,10 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="1" t="n">
-        <v>45657</v>
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2024-12-31</t>
+        </is>
       </c>
       <c r="B127" t="n">
         <v>0.06</v>
@@ -17910,8 +18158,10 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="1" t="n">
-        <v>45688</v>
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2025-01-31</t>
+        </is>
       </c>
       <c r="B128" t="n">
         <v>0.06</v>
@@ -18047,8 +18297,10 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="1" t="n">
-        <v>45716</v>
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2025-02-28</t>
+        </is>
       </c>
       <c r="B129" t="n">
         <v>0</v>
@@ -18184,8 +18436,10 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="1" t="n">
-        <v>45747</v>
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
       </c>
       <c r="B130" t="n">
         <v>0</v>
@@ -18321,8 +18575,10 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="1" t="n">
-        <v>45777</v>
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2025-04-30</t>
+        </is>
       </c>
       <c r="B131" t="n">
         <v>0.2425</v>
@@ -18458,8 +18714,10 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="1" t="n">
-        <v>45838</v>
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2025-06-30</t>
+        </is>
       </c>
       <c r="B132" t="n">
         <v>0.2651</v>
@@ -18595,8 +18853,10 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="1" t="n">
-        <v>45869</v>
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2025-07-31</t>
+        </is>
       </c>
       <c r="B133" t="n">
         <v>0.06</v>
@@ -18732,8 +18992,10 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" s="1" t="n">
-        <v>45930</v>
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2025-09-30</t>
+        </is>
       </c>
       <c r="B134" t="n">
         <v>0</v>
@@ -18869,8 +19131,10 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="1" t="n">
-        <v>45961</v>
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2025-10-31</t>
+        </is>
       </c>
       <c r="B135" t="n">
         <v>0</v>
@@ -19006,8 +19270,10 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="1" t="n">
-        <v>46022</v>
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
       </c>
       <c r="B136" t="n">
         <v>0</v>
@@ -19143,8 +19409,10 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="1" t="n">
-        <v>46112</v>
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
       </c>
       <c r="B137" t="n">
         <v>0.15</v>
@@ -19280,8 +19548,10 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="1" t="n">
-        <v>46142</v>
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
       </c>
       <c r="B138" t="n">
         <v>0.2662</v>

</xml_diff>